<commit_message>
Añadir nuevo grupo y sub servicios a recargas
</commit_message>
<xml_diff>
--- a/src/recargas/cuentas.xlsx
+++ b/src/recargas/cuentas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\TeamComunicaciones\automatizadorteam\src\recargas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\corte\poliedro\IntegrateamCode\src\recargas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C44CFB-CC3B-4FD0-A470-C6735CFB8E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="4530" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19170" yWindow="1210" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,6 +59,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -405,12 +406,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -418,7 +419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -426,7 +427,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -434,7 +435,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -442,7 +443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -450,7 +451,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -458,31 +459,31 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Agregar dos codigos de distribuidor al modulo de poliedro
</commit_message>
<xml_diff>
--- a/src/recargas/cuentas.xlsx
+++ b/src/recargas/cuentas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\corte\poliedro\IntegrateamCode\src\recargas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C44CFB-CC3B-4FD0-A470-C6735CFB8E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78661C3E-5D0D-4336-84BE-5EF84A2AF03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19170" yWindow="1210" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
     <t>cuenta</t>
   </si>
   <si>
-    <t>aux1</t>
-  </si>
-  <si>
     <t>aux2</t>
   </si>
   <si>
@@ -41,6 +38,9 @@
   </si>
   <si>
     <t>aux5</t>
+  </si>
+  <si>
+    <t>3810000002</t>
   </si>
 </sst>
 </file>
@@ -97,12 +97,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,73 +424,76 @@
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>2</v>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
+      <c r="B3" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
+      <c r="B4" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>6</v>
+      <c r="B6" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="2"/>
+      <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="2"/>
+      <c r="B9" s="3"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="2"/>
+      <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="B11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError sqref="B2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Recargas: grupo/servicio dinamicos por scraping + ajustes layout PRE-SIM
Funcionalidad 2 (recargas):
- scraper_catalogo_recargas.py: lee la relacion grupo->servicios del portal
  (por texto, ids Angular cambian); no realiza recargas.
- catalogo_recargas.py: lee/escribe catalogo.xlsx (archivo aparte, formato
  grupo|servicio) y expone el mapa dependiente.
- recargas.py: quita listas hardcodeadas; combos Grupo/Servicio dinamicos y
  dependientes desde el catalogo; boton "ACTUALIZAR LISTAS" que scrapea (login
  con 1a cuenta + Clave UI, navegador visible) y regenera el catalogo.
- combobox.py: soporta command (callback al cambiar) para la dependencia.
- sub_menu.py: alto parametrizable (default 0.74, no afecta otros modulos).

Ajustes Funcionalidad 1 (PRE-SIM):
- mixin_validacion_codigos.py: checkbox de validacion admite place opcional.
- preactivador.py: recompactado del panel para que el checkbox no tape el correo.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/recargas/cuentas.xlsx
+++ b/src/recargas/cuentas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\corte\poliedro\IntegrateamCode\src\recargas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78661C3E-5D0D-4336-84BE-5EF84A2AF03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FEEF54A-508C-4E92-BBA8-26E3B601255C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <t>aux5</t>
   </si>
   <si>
-    <t>3810000002</t>
+    <t>16USUARIO</t>
   </si>
 </sst>
 </file>
@@ -492,8 +492,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="B2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>